<commit_message>
Actualizar Banco General de Preguntas
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -505,6 +505,1466 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PAT_00001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Caída de cabello (Alopecia)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Caída de cabello (Alopecia).</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Espolón calcáneo / dolor de talón (fascitis plantar asociada)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Androgenética (DHT)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Insomnio</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Se relaciona con Disminución de densidad</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PAT_00002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Salud prostática / Molestias prostáticas</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Salud prostática / Molestias prostáticas.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Se relaciona con Chorro débil</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Dolor muscular, contracturas y molestias musculoesqueléticas localizadas</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Hiperplasia prostática benigna</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Quistes ováricos funcionales</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PAT_00003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Disfunción sexual masculina / Dificultad para la erección.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Estrés o ansiedad</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Perimenopausia / Menopausia</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Endometriosis</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Se relaciona con Disminución de la libido</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PAT_00004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Vitalidad masculina y apoyo hormonal (Hipogonadismo / Deficiencia de testosterona*)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Vitalidad masculina y apoyo hormonal (Hipogonadismo / Deficiencia de testosterona*).</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Ciática / Lumbalgia</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Se relaciona con Disminución de la libido</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Envejecimiento</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Insomnio</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2,3</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PAT_00005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Control glucémico (Diabetes mellitus tipo 2 / Prediabetes)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Control glucémico (Diabetes mellitus tipo 2 / Prediabetes).</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Se relaciona con Diagnóstico de diabetes o prediabetes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Resistencia a la insulina</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Artritis inflamatoria</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Quistes ováricos funcionales</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PAT_00006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Perimenopausia / Menopausia</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Perimenopausia / Menopausia.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Se relaciona con Alteraciones menstruales</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Disminución fisiológica de estrógenos y progesterona</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Espolón calcáneo / dolor de talón (fascitis plantar asociada)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Insomnio</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>P006</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PAT_00007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Insomnio</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Insomnio.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Ciática / Lumbalgia</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Estrés</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dificultad para conciliar el sueño</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Osteoporosis</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2,3</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>P007</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PAT_00008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Varicocele (Apoyo a la salud vascular y reproductiva masculina)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Varicocele (Apoyo a la salud vascular y reproductiva masculina).</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Insuficiencia de las válvulas venosas del cordón espermático</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Se relaciona con Diagnóstico médico de varicocele</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Perimenopausia / Menopausia</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2,3</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>P008</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PAT_00009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bienestar íntimo femenino y función sexual</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Bienestar íntimo femenino y función sexual.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Disminución de estrógenos (perimenopausia/menopausia)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Se relaciona con Disminución de la libido</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Síndrome de Ovario Poliquístico (SOP)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>P009</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PAT_00010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Apoyo a la salud reproductiva femenina y planificación del embarazo</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Apoyo a la salud reproductiva femenina y planificación del embarazo.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Bienestar íntimo femenino y función sexual</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dificultad para lograr embarazo</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Perimenopausia / Menopausia</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Déficit nutricional (ácido fólico, hierro, zinc, vitamina D)</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>P010</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PAT_00011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Síndrome de Ovario Poliquístico (SOP)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Síndrome de Ovario Poliquístico (SOP).</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Se relaciona con Menstruaciones irregulares o ausencia de menstruación</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Varicocele (Apoyo a la salud vascular y reproductiva masculina)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Artritis inflamatoria</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Predisposición genética</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>P011</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PAT_00012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Quistes ováricos funcionales</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Quistes ováricos funcionales.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor pélvico unilateral</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Cambios normales del ciclo ovulatorio</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Salud prostática / Molestias prostáticas</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>P012</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PAT_00013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Endometriosis</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Endometriosis.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Salud prostática / Molestias prostáticas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Artritis inflamatoria</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Predisposición genética</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor menstrual intenso</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>P013</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PAT_00014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Osteoporosis</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Osteoporosis.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Síndrome de Ovario Poliquístico (SOP)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Envejecimiento</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Salud prostática / Molestias prostáticas</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor de espalda frecuente</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>P014</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PAT_00015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Artrosis (desgaste articular / osteoartritis)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Artrosis (desgaste articular / osteoartritis).</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Dolor muscular, contracturas y molestias musculoesqueléticas localizadas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Envejecimiento</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Ciática / Lumbalgia</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor en rodillas, cadera, manos o columna</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>P015</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PAT_00016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Artritis inflamatoria</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Artritis inflamatoria.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor articular</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Síndrome de Ovario Poliquístico (SOP)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Alteraciones del sistema inmunológico</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>P016</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PAT_00017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ciática / Lumbalgia</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Ciática / Lumbalgia.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Bienestar íntimo femenino y función sexual</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor lumbar</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Sobrecarga física</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>P017</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PAT_00018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dolor muscular, contracturas y molestias musculoesqueléticas localizadas</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Dolor muscular, contracturas y molestias musculoesqueléticas localizadas.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Disfunción sexual masculina / Dificultad para la erección</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Salud prostática / Molestias prostáticas</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Esfuerzo físico</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor localizado</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>P018</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PAT_00019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Fibromialgia</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Fibromialgia.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor generalizado en diferentes zonas del cuerpo</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Espolón calcáneo / dolor de talón (fascitis plantar asociada)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Alteraciones en la percepción del dolor</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Dolor muscular, contracturas y molestias musculoesqueléticas localizadas</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>P019</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PAT_00020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Patologias</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Espolón calcáneo / dolor de talón (fascitis plantar asociada)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sintoma_Causa_Patologia</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Seleccione las DOS afirmaciones que se relacionan correctamente con Espolón calcáneo / dolor de talón (fascitis plantar asociada).</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Se relaciona con Dolor en el talón al dar los primeros pasos</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Puede estar asociada a Sobrecarga del pie</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Se relaciona principalmente con Control glucémico (Diabetes mellitus tipo 2 / Prediabetes)</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Puede estar asociada principalmente a Perimenopausia / Menopausia</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-08-18 21:59:11</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>P020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar estados Banco General
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -636,7 +636,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -709,7 +709,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -782,7 +782,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
@@ -2899,7 +2899,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
@@ -3264,7 +3264,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -3556,7 +3556,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M45" t="inlineStr"/>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M46" t="inlineStr"/>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M48" t="inlineStr"/>
@@ -3994,7 +3994,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M49" t="inlineStr"/>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M50" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M51" t="inlineStr"/>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M52" t="inlineStr"/>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M53" t="inlineStr"/>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M54" t="inlineStr"/>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M55" t="inlineStr"/>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M56" t="inlineStr"/>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M57" t="inlineStr"/>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M58" t="inlineStr"/>
@@ -4724,7 +4724,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M59" t="inlineStr"/>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M60" t="inlineStr"/>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M61" t="inlineStr"/>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M62" t="inlineStr"/>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M63" t="inlineStr"/>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M64" t="inlineStr"/>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M65" t="inlineStr"/>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M66" t="inlineStr"/>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M67" t="inlineStr"/>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M68" t="inlineStr"/>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M69" t="inlineStr"/>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M70" t="inlineStr"/>
@@ -5600,7 +5600,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M71" t="inlineStr"/>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M72" t="inlineStr"/>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M73" t="inlineStr"/>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M74" t="inlineStr"/>
@@ -5892,7 +5892,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M75" t="inlineStr"/>
@@ -5965,7 +5965,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M76" t="inlineStr"/>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M77" t="inlineStr"/>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M78" t="inlineStr"/>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M79" t="inlineStr"/>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M80" t="inlineStr"/>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M81" t="inlineStr"/>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M82" t="inlineStr"/>
@@ -6476,7 +6476,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M83" t="inlineStr"/>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M84" t="inlineStr"/>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M85" t="inlineStr"/>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M86" t="inlineStr"/>
@@ -6768,7 +6768,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M87" t="inlineStr"/>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M88" t="inlineStr"/>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M89" t="inlineStr"/>
@@ -6987,7 +6987,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M90" t="inlineStr"/>
@@ -7060,7 +7060,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M91" t="inlineStr"/>
@@ -7133,7 +7133,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M92" t="inlineStr"/>
@@ -7206,7 +7206,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M93" t="inlineStr"/>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M94" t="inlineStr"/>
@@ -7352,7 +7352,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M95" t="inlineStr"/>
@@ -7425,7 +7425,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M96" t="inlineStr"/>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M97" t="inlineStr"/>
@@ -7571,7 +7571,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M98" t="inlineStr"/>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M99" t="inlineStr"/>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M100" t="inlineStr"/>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M101" t="inlineStr"/>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M102" t="inlineStr"/>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M103" t="inlineStr"/>
@@ -8009,7 +8009,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M104" t="inlineStr"/>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M105" t="inlineStr"/>
@@ -8155,7 +8155,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M106" t="inlineStr"/>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M107" t="inlineStr"/>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M108" t="inlineStr"/>
@@ -8374,7 +8374,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M109" t="inlineStr"/>
@@ -8447,7 +8447,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M110" t="inlineStr"/>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M111" t="inlineStr"/>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M112" t="inlineStr"/>
@@ -8666,7 +8666,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M113" t="inlineStr"/>
@@ -8739,7 +8739,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M114" t="inlineStr"/>
@@ -8812,7 +8812,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M115" t="inlineStr"/>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M116" t="inlineStr"/>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M117" t="inlineStr"/>
@@ -9031,7 +9031,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M118" t="inlineStr"/>
@@ -9104,7 +9104,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M119" t="inlineStr"/>
@@ -9177,7 +9177,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M120" t="inlineStr"/>
@@ -9250,7 +9250,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M121" t="inlineStr"/>
@@ -9323,7 +9323,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M122" t="inlineStr"/>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M123" t="inlineStr"/>
@@ -9469,7 +9469,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M124" t="inlineStr"/>
@@ -9542,7 +9542,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M125" t="inlineStr"/>
@@ -9615,7 +9615,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M126" t="inlineStr"/>
@@ -9688,7 +9688,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M127" t="inlineStr"/>
@@ -9761,7 +9761,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M128" t="inlineStr"/>
@@ -9834,7 +9834,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M129" t="inlineStr"/>
@@ -9907,7 +9907,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M130" t="inlineStr"/>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M131" t="inlineStr"/>
@@ -10053,7 +10053,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M132" t="inlineStr"/>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M133" t="inlineStr"/>
@@ -10199,7 +10199,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M134" t="inlineStr"/>
@@ -10272,7 +10272,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M135" t="inlineStr"/>
@@ -10345,7 +10345,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M136" t="inlineStr"/>
@@ -10418,7 +10418,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M137" t="inlineStr"/>
@@ -10491,7 +10491,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M138" t="inlineStr"/>
@@ -10564,7 +10564,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M139" t="inlineStr"/>
@@ -10637,7 +10637,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M140" t="inlineStr"/>
@@ -10710,7 +10710,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M141" t="inlineStr"/>
@@ -10783,7 +10783,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M142" t="inlineStr"/>
@@ -10856,7 +10856,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M143" t="inlineStr"/>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M144" t="inlineStr"/>
@@ -11002,7 +11002,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M145" t="inlineStr"/>
@@ -11075,7 +11075,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M146" t="inlineStr"/>
@@ -11148,7 +11148,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M147" t="inlineStr"/>
@@ -11221,7 +11221,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M148" t="inlineStr"/>
@@ -11294,7 +11294,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M149" t="inlineStr"/>
@@ -11367,7 +11367,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M150" t="inlineStr"/>
@@ -11440,7 +11440,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M151" t="inlineStr"/>
@@ -11513,7 +11513,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M152" t="inlineStr"/>
@@ -11586,7 +11586,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M153" t="inlineStr"/>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M154" t="inlineStr"/>
@@ -11732,7 +11732,7 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M155" t="inlineStr"/>
@@ -11805,7 +11805,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M156" t="inlineStr"/>
@@ -11878,7 +11878,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M157" t="inlineStr"/>
@@ -11951,7 +11951,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M158" t="inlineStr"/>
@@ -12024,7 +12024,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M159" t="inlineStr"/>
@@ -12097,7 +12097,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M160" t="inlineStr"/>
@@ -12170,7 +12170,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="M161" t="inlineStr"/>

</xml_diff>

<commit_message>
Generar preguntas de Restricciones
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O166"/>
+  <dimension ref="A1:O171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12550,6 +12550,371 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>RES_00006</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>FITO OMEGA 3</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Producto_Motivo</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO OMEGA 3. Seleccione las DOS afirmaciones que corresponden a información registrada para sus restricciones.</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: Los laxantes estimulantes pueden irritar el colon y agravar estas condiciones..</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: La coenzima Q10 puede interferir con el efecto anticoagulante de algunos medicamentos..</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>El motivo indicado es: Producto de origen marino..</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Otro motivo registrado para este producto es: Puede incrementar el riesgo de sangrado..</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr"/>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>2026-08-19 00:36:30</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>X007</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>RES_00007</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>FITO OMEGA 3</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Producto_Motivo</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO OMEGA 3. Seleccione las DOS afirmaciones que corresponden a información registrada para sus restricciones.</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>El motivo indicado es: Puede incrementar el riesgo de sangrado..</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Otro motivo registrado para este producto es: Producto de origen marino..</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: La disminución de la función renal puede favorecer la acumulación de magnesio..</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: La suplementación debe individualizarse en personas con alteración renal..</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>2026-08-19 00:36:30</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>X008</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>RES_00008</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>FITO COLÁGENO MARINO PLUS</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Producto_Motivo</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO COLÁGENO MARINO PLUS. Seleccione las DOS afirmaciones que corresponden a información registrada para sus restricciones.</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>El motivo indicado es: Contiene colágeno de origen marino..</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: Puede incrementar el riesgo de sangrado..</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: La L-Arginina favorece la vasodilatación y puede potenciar la disminución de la presión arterial..</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Otro motivo registrado para este producto es: Contiene colágeno de origen marino..</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr"/>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>2026-08-19 00:36:30</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>X009</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>RES_00009</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>OSHECAL</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Producto_Motivo</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Considere el producto OSHECAL. Seleccione las DOS afirmaciones que corresponden a información registrada para sus restricciones.</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: La valeriana puede potenciar el efecto sedante de otros medicamentos o sustancias depresoras del sistema nervioso central, aumentando la somnolencia..</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: La vitamina E en dosis suplementarias puede aumentar el riesgo de sangrado en personas con medicamentos que afectan la coagulación..</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Otro motivo registrado para este producto es: La suplementación con calcio debe individualizarse cuando existen alteraciones en eliminación renal o manejo del calcio..</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>El motivo indicado es: Al ser un producto en polvo/multivitamínico puede contener componentes que deben revisarse según la formulación y el control nutricional del usuario..</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>2026-08-19 00:36:30</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>X019</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>RES_00010</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>OSHECAL</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Nivel 2</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Producto_Motivo</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Considere el producto OSHECAL. Seleccione las DOS afirmaciones que corresponden a información registrada para sus restricciones.</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: Su aporte elevado de calorías puede favorecer aumento de peso no deseado si no existe demanda energética o entrenamiento..</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>El motivo registrado es: Es un producto orientado al control de peso y no debe utilizarse en personas donde la pérdida de peso no sea apropiada..</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Otro motivo registrado para este producto es: Al ser un producto en polvo/multivitamínico puede contener componentes que deben revisarse según la formulación y el control nutricional del usuario..</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>El motivo indicado es: La suplementación con calcio debe individualizarse cuando existen alteraciones en eliminación renal o manejo del calcio..</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>2026-08-19 00:36:30</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>X020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar preguntas Producto - Accion General
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O176"/>
+  <dimension ref="A1:O181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13280,6 +13280,371 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>PROD_00001</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>OREGANO OIL x 150 SOFTGELS</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Producto_AccionGeneral</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Considere el producto OREGANO OIL x 150 SOFTGELS. ¿Cuál de las siguientes acciones generales corresponde a este producto según la matriz?</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>MODO DE ACCIÓN: acción antifúngica y antibacteriana potente al alterar membrana celular de hongos y bacterias</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Artrifit (dolor reumático)</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Gel de Caléndula (apoyo tópico en piel irritada)</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Apoyo en regulación emocional en personas hipersensibles</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>RECHAZADA</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>2026-08-19 20:26:46</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>oregano oil x 150 softgels||modo de acción: acción antifúngica y antibacteriana potente al alterar membrana celular de hongos y bacterias</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>PROD_00002</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>FITO GEL DE CALENDULA x 300 GR</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Producto_AccionGeneral</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO GEL DE CALENDULA x 300 GR. ¿Cuál de las siguientes acciones generales corresponde a este producto según la matriz?</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Apoyo en expulsión de flema ligera</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>flor de jamaica con apoyo diurético suave y antioxidante, útil en retención de líquidos. Puede apoyar digestión y sensación de pesadez. COMBINACIONES: Dunplus (pérdida de peso/metabolismo)</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>yantén como calmante tradicional. Gel frío con efecto refrescante que disminuye sensación de ardor e inflamación. Apoyo en regeneración cutánea en quemaduras leves y lesiones superficiales (coadyuvante). COMBINACIONES: Castaño de Indias cápsulas (circulación interna + externa)</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Cloruro de Magnesio (apoyo muscular)</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>RECHAZADA</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>2026-08-19 20:26:46</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>fito gel de calendula x 300 gr||yantén como calmante tradicional. gel frío con efecto refrescante que disminuye sensación de ardor e inflamación. apoyo en regeneración cutánea en quemaduras leves y lesiones superficiales (coadyuvante). combinaciones: castaño de indias cápsulas (circulación interna + externa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>PROD_00003</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>FITO ARTRIFIT x 60 CAP</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Producto_AccionGeneral</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO ARTRIFIT x 60 CAP. ¿Cuál de las siguientes acciones generales corresponde a este producto según la matriz?</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Magnesio (sistema nervioso)</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Mejora rigidez y movilidad</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Zinc adicional (defensas). FRASE DE VENTA: 'Ayuda a descongestionar y reforzar defensas en gripa con mocos.'</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>apoyo en oxigenación cerebral</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>RECHAZADA</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>2026-08-19 20:26:46</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>fito artrifit x 60 cap||mejora rigidez y movilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>PROD_00004</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>FITO OMEGA 3 x 100 PERLAS</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Producto_AccionGeneral</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO OMEGA 3 x 100 PERLAS. ¿Cuál de las siguientes acciones generales corresponde a este producto según la matriz?</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>apoyo antioxidante</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Biotina (cabello si hay déficit). FRASE DE VENTA: 'Detox verde completo: limpia, nutre, energiza y fortalece defensas.'</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Vitamina E cosmética (piel seca). FRASE DE VENTA: 'Calma y regenera tu piel de forma natural.'</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Colágeno Marino (articulaciones/piel)</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>RECHAZADA</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>2026-08-19 20:26:46</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>fito omega 3 x 100 perlas||colágeno marino (articulaciones/piel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>PROD_00005</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>FITO GINKGO BILOBA x 100 CAP</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Producto_AccionGeneral</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Considere el producto FITO GINKGO BILOBA x 100 CAP. ¿Cuál de las siguientes acciones generales corresponde a este producto según la matriz?</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>apoyo indirecto en dolor articular leve asociado a componente circulatorio. COMBINACIONES: Breinap (memoria + energía mental)</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Nutrición de fibra capilar y piel</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>apoyo en piel (regulación de inflamación y sebo, acné)</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Apoyo en conciliación del sueño cuando hay nerviosismo</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>RECHAZADA</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>2026-08-19 20:26:46</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>fito ginkgo biloba x 100 cap||apoyo indirecto en dolor articular leve asociado a componente circulatorio. combinaciones: breinap (memoria + energía mental)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar preguntas aprobadas 7.7
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -14534,42 +14534,42 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Causas</t>
+          <t>Condición - Producto + Coadyuvantes</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Nivel 1</t>
+          <t>Nivel 2</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Patología-Causas</t>
+          <t>Patología-Condición-Producto-Coadyuvantes</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>¿Cuál de las siguientes opciones corresponde a las causas frecuentes de la patología Espolón calcáneo / dolor de talón (fascitis plantar asociada)?</t>
+          <t>Para la patología Varicocele (Apoyo a la salud vascular y reproductiva masculina), si se presenta el perfil o condición Varicocele sin complicaciones asociadas, ¿cuál sería el paquete recomendado?</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Predisposición genética; resistencia a la insulina; sobrepeso u obesidad; alteraciones hormonales; inflamación crónica de bajo grado; sedentarismo; factores ambientales.</t>
+          <t>INOSITOL (Terceros) | BERBERINA (Terceros); CROMO (Terceros)</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Sobrecarga del pie; aumento de peso; estar mucho tiempo de pie; actividad física intensa; calzado inadecuado; alteraciones de apoyo plantar; envejecimiento.</t>
+          <t>FITO CASTAÑO DE INDIAS | FITO OMEGA 3</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Androgenética (DHT); déficit nutricional (hierro/zinc/biotina/proteína); estrés y alteración del sueño; postparto; perimenopausia/menopausia; cuero cabelludo (caspa/dermatitis); fármacos/quimio; químicos/cosméticos; tiroides.</t>
+          <t>ARTRIFIT | Cloruro de Magnesio; CALGEL</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>Predisposición genética; menstruación retrógrada; alteraciones inmunológicas; factores hormonales; inflamación crónica.</t>
+          <t>FITO GLOBXAN | Ninguno</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -14585,12 +14585,12 @@
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr">
         <is>
-          <t>2026-08-23 18:01:44</t>
+          <t>2026-08-23 20:13:38</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>PTG-F000020</t>
+          <t>P008</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar preguntas 7.8 - Complementarios
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O198"/>
+  <dimension ref="A1:O199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14886,6 +14886,79 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>PTCOM-000001</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Complementarios</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Producto-Indicaciones-Combinaciones</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>El producto Zarzaparrilla usualmente se recomienda para Acné hormonal; Problemas cutáneos crónicos; Inflamación leve; Retención de líquidos leve; Artritis leve (apoyo). ¿Cuál de las siguientes opciones corresponde a la combinación estratégica recomendada?</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Isowoan; Zinc; L-Arginina; Creatina; Proteína; Ashwagandha</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Alcachofa (detox piel); Orégano (acné inflamatorio); Isowoan (mujer hormonal)</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Proteína; Creatina</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Fibra; Biotics</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>APROBADA</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr"/>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>2026-08-23 21:05:42</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>COM-F000002</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar preguntas 8.1 - Restricciones
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O199"/>
+  <dimension ref="A1:O200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14959,6 +14959,79 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>PTRX-000001</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Precaución / Contraindicación</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Producto-Precaución/Contraindicación</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Para el producto CLORURO DE MAGNESIO, ¿cuál de las siguientes corresponde a una precaución o contraindicación para su uso?</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Insuficiencia renal moderada o severa; hipermagnesemia diagnosticada.</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Uso de warfarina u otros anticoagulantes</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Insuficiencia renal moderada o avanzada; hipermagnesemia</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Persona sedentaria cuyo objetivo es únicamente osteoporosis sin pérdida de masa muscular identificada</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>APROBADA</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr"/>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>2026-08-23 21:39:44</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>RX-000043</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar preguntas 8.2 - Producto Contraindicación Motivo
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O202"/>
+  <dimension ref="A1:O203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15178,6 +15178,79 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>PTRM-000001</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Producto / Contraindicación - Motivo</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Producto-Precaución/Contraindicación-Motivo</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>FITO VITAMINA D3 puede generar contraindicaciones asociadas a Hipercalcemia, antecedentes de exceso de vitamina D o enfermedades que alteren metabolismo del calcio debido a que:</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>La suplementación con calcio debe individualizarse cuando existen alteraciones en eliminación renal o manejo del calcio.</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>La vitamina D aumenta la absorción de calcio y debe ajustarse cuando hay alteraciones del metabolismo mineral.</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>El resveratrol puede presentar efecto modulador sobre la agregación plaquetaria y requiere precaución en personas con riesgo de sangrado.</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>La vitamina E en dosis suplementarias puede aumentar el riesgo de sangrado en personas con medicamentos que afectan la coagulación.</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>APROBADA</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr"/>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>2026-08-24 14:34:38</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>X027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar preguntas 8.3 - Producto Restricción Alternativas Seguras
</commit_message>
<xml_diff>
--- a/BANCO_PREGUNTAS_GENERALES.xlsx
+++ b/BANCO_PREGUNTAS_GENERALES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O203"/>
+  <dimension ref="A1:O204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15251,6 +15251,79 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>PTRS-000003</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Restricciones</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Producto / Alternativas seguras</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Nivel 1</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Producto-Alternativas seguras</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Para el producto FITO MELATONINA, ¿cuál de las siguientes corresponde a una alternativa segura?</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>FITO ESENCIA FLORAL INSOMNIO; medidas de higiene del sueño; valoración médica cuando el insomnio sea persistente.</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>FITO VITAMINA D3; FITO CLORURO DE MAGNESIO (según objetivo)</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>FITO RESVERATROL o antioxidantes alternativos según perfil</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Recomendar valoración médica antes de aumentar el consumo de proteínas.</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>APROBADA</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr"/>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>2026-08-24 15:03:39</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>X017</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>